<commit_message>
Implementación de tablas de precios y términos de contrato. Se implementaron también la mayoría de los reportes. Dashboard está a un 70%.
</commit_message>
<xml_diff>
--- a/liquidacion_complejo.xlsx
+++ b/liquidacion_complejo.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="102">
   <si>
     <t xml:space="preserve">LIQUIDACIÓN DEL MINERAL Pb - Ag - Zn - BROZA</t>
   </si>
@@ -390,6 +390,12 @@
   </si>
   <si>
     <t xml:space="preserve">SACOS:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cot Ag Tn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VNV Ag $us</t>
   </si>
   <si>
     <t xml:space="preserve">ADMINISTRACION</t>
@@ -898,7 +904,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="125">
+  <cellXfs count="126">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1396,6 +1402,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4210,20 +4220,20 @@
     </row>
     <row r="15" customFormat="false" ht="12.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="25" t="n">
-        <v>6100</v>
+        <v>1000</v>
       </c>
       <c r="C15" s="26" t="n">
         <v>0</v>
       </c>
       <c r="D15" s="26" t="n">
-        <v>2.3</v>
+        <v>0</v>
       </c>
       <c r="E15" s="26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F15" s="27" t="n">
         <f aca="false">(B15-C15)*(1-D15/100)*(1-E15/100)</f>
-        <v>5900.103</v>
+        <v>1000</v>
       </c>
       <c r="G15" s="28" t="s">
         <v>20</v>
@@ -4236,7 +4246,7 @@
       </c>
       <c r="J15" s="31" t="n">
         <f aca="false">F15*H15/100</f>
-        <v>649.01133</v>
+        <v>110</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4256,7 +4266,7 @@
       </c>
       <c r="J16" s="31" t="n">
         <f aca="false">F15*H16/100</f>
-        <v>1298.02266</v>
+        <v>220</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4265,14 +4275,14 @@
         <v>23</v>
       </c>
       <c r="H17" s="123" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="I17" s="36" t="s">
         <v>24</v>
       </c>
       <c r="J17" s="37" t="n">
         <f aca="false">F15/1000*H17*100/1000</f>
-        <v>19.4703399</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4284,7 +4294,7 @@
       <c r="I18" s="39"/>
       <c r="J18" s="40" t="n">
         <f aca="false">SUM(J15:J17)</f>
-        <v>1966.5043299</v>
+        <v>333.5</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="5.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4357,26 +4367,26 @@
       </c>
       <c r="F23" s="48" t="n">
         <f aca="false">J15/1000*2204.6223*D23</f>
-        <v>2289.31976171305</v>
+        <v>388.0135248</v>
       </c>
       <c r="G23" s="49" t="n">
         <f aca="false">F23*D$11</f>
-        <v>15933.6655415229</v>
+        <v>2700.574132608</v>
       </c>
       <c r="H23" s="46" t="n">
         <v>3</v>
       </c>
       <c r="I23" s="48" t="n">
         <f aca="false">F23*H23/100</f>
-        <v>68.6795928513916</v>
+        <v>11.640405744</v>
       </c>
       <c r="J23" s="48" t="n">
         <f aca="false">I23*D$11</f>
-        <v>478.009966245686</v>
+        <v>81.01722397824</v>
       </c>
       <c r="K23" s="50" t="n">
         <f aca="false">G23*H23/100</f>
-        <v>478.009966245686</v>
+        <v>81.01722397824</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4392,26 +4402,26 @@
       </c>
       <c r="F24" s="48" t="n">
         <f aca="false">J16/1000*2204.6223*D24</f>
-        <v>2575.48473192719</v>
+        <v>436.5152154</v>
       </c>
       <c r="G24" s="49" t="n">
         <f aca="false">F24*D$11</f>
-        <v>17925.3737342132</v>
+        <v>3038.145899184</v>
       </c>
       <c r="H24" s="46" t="n">
         <v>3</v>
       </c>
       <c r="I24" s="48" t="n">
         <f aca="false">F24*H24/100</f>
-        <v>77.2645419578156</v>
+        <v>13.095456462</v>
       </c>
       <c r="J24" s="48" t="n">
         <f aca="false">I24*D$11</f>
-        <v>537.761212026397</v>
+        <v>91.14437697552</v>
       </c>
       <c r="K24" s="50" t="n">
         <f aca="false">G24*H24/100</f>
-        <v>537.761212026397</v>
+        <v>91.14437697552</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4427,26 +4437,26 @@
       </c>
       <c r="F25" s="48" t="n">
         <f aca="false">J17*1000/31.1035*D25</f>
-        <v>47117.9283448165</v>
+        <v>8469.94711206134</v>
       </c>
       <c r="G25" s="49" t="n">
         <f aca="false">F25*D$11</f>
-        <v>327940.781279923</v>
+        <v>58950.831899947</v>
       </c>
       <c r="H25" s="46" t="n">
         <v>3.6</v>
       </c>
       <c r="I25" s="48" t="n">
         <f aca="false">F25*H25/100</f>
-        <v>1696.24542041339</v>
+        <v>304.918096034208</v>
       </c>
       <c r="J25" s="48" t="n">
         <f aca="false">I25*D$11</f>
-        <v>11805.8681260772</v>
+        <v>2122.22994839809</v>
       </c>
       <c r="K25" s="50" t="n">
         <f aca="false">G25*H25/100</f>
-        <v>11805.8681260772</v>
+        <v>2122.22994839809</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4456,24 +4466,24 @@
       </c>
       <c r="F26" s="124" t="n">
         <f aca="false">SUM(F23:F25)</f>
-        <v>51982.7328384567</v>
+        <v>9294.47585226134</v>
       </c>
       <c r="G26" s="49" t="n">
         <f aca="false">SUM(G23:G25)</f>
-        <v>361799.820555659</v>
+        <v>64689.551931739</v>
       </c>
       <c r="H26" s="51"/>
       <c r="I26" s="52" t="n">
         <f aca="false">SUM(I23:I25)</f>
-        <v>1842.1895552226</v>
+        <v>329.653958240208</v>
       </c>
       <c r="J26" s="52" t="n">
         <f aca="false">SUM(J23:J25)</f>
-        <v>12821.6393043493</v>
+        <v>2294.39154935185</v>
       </c>
       <c r="K26" s="50" t="n">
         <f aca="false">SUM(K23:K25)</f>
-        <v>12821.6393043493</v>
+        <v>2294.39154935185</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="5.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4526,7 +4536,14 @@
       <c r="E30" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="I30" s="33"/>
+      <c r="G30" s="1" t="n">
+        <f aca="false">1000*1000/31.1035</f>
+        <v>32150.7225874902</v>
+      </c>
+      <c r="I30" s="33" t="n">
+        <f aca="false">H17/10000*G33</f>
+        <v>4202.90321024965</v>
+      </c>
       <c r="J30" s="44"/>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4541,7 +4558,7 @@
       </c>
       <c r="E31" s="48" t="n">
         <f aca="false">J15/1000*2204.6223*C31</f>
-        <v>1787.38640395747</v>
+        <v>302.9415594876</v>
       </c>
       <c r="I31" s="33"/>
       <c r="J31" s="44"/>
@@ -4558,7 +4575,13 @@
       </c>
       <c r="E32" s="48" t="n">
         <f aca="false">J16/1000*2204.6223*C32</f>
-        <v>2490.20757080337</v>
+        <v>422.0617116012</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>94</v>
       </c>
       <c r="I32" s="33"/>
       <c r="J32" s="44"/>
@@ -4573,9 +4596,17 @@
       <c r="D33" s="47" t="s">
         <v>36</v>
       </c>
-      <c r="E33" s="48" t="e">
-        <f aca="false">J17*1000/31.1035*c33j17j17</f>
-        <v>#NAME?</v>
+      <c r="E33" s="48" t="n">
+        <f aca="false">J17*1000/31.1035*C33</f>
+        <v>4202.90321024965</v>
+      </c>
+      <c r="G33" s="125" t="n">
+        <f aca="false">C33*1000*1000/31.1035</f>
+        <v>1200829.48864276</v>
+      </c>
+      <c r="H33" s="125" t="n">
+        <f aca="false">G33*J17/1000</f>
+        <v>4202.90321024965</v>
       </c>
       <c r="J33" s="61"/>
     </row>
@@ -4584,9 +4615,9 @@
         <v>41</v>
       </c>
       <c r="C34" s="63"/>
-      <c r="D34" s="64" t="e">
+      <c r="D34" s="64" t="n">
         <f aca="false">SUM(E31:E33)</f>
-        <v>#NAME?</v>
+        <v>4927.90648133845</v>
       </c>
       <c r="E34" s="65" t="s">
         <v>42</v>
@@ -4600,9 +4631,9 @@
         <v>41</v>
       </c>
       <c r="C35" s="68"/>
-      <c r="D35" s="69" t="e">
+      <c r="D35" s="69" t="n">
         <f aca="false">D34*D11</f>
-        <v>#NAME?</v>
+        <v>34298.2291101156</v>
       </c>
       <c r="E35" s="70" t="s">
         <v>43</v>
@@ -4653,7 +4684,7 @@
       <c r="C38" s="63"/>
       <c r="D38" s="64" t="n">
         <f aca="false">D37*F15/1000</f>
-        <v>11800.206</v>
+        <v>2000</v>
       </c>
       <c r="E38" s="62" t="s">
         <v>49</v>
@@ -4671,7 +4702,7 @@
       <c r="C39" s="68"/>
       <c r="D39" s="80" t="n">
         <f aca="false">D38*D11</f>
-        <v>82129.43376</v>
+        <v>13920</v>
       </c>
       <c r="E39" s="81" t="s">
         <v>43</v>
@@ -4707,7 +4738,7 @@
       </c>
       <c r="G41" s="87" t="n">
         <f aca="false">J26</f>
-        <v>12821.6393043493</v>
+        <v>2294.39154935185</v>
       </c>
       <c r="H41" s="62" t="s">
         <v>53</v>
@@ -4731,7 +4762,7 @@
       </c>
       <c r="G42" s="88" t="n">
         <f aca="false">D39*D42/100</f>
-        <v>1478.32980768</v>
+        <v>250.56</v>
       </c>
       <c r="H42" s="62" t="s">
         <v>53</v>
@@ -4754,7 +4785,7 @@
       </c>
       <c r="G43" s="88" t="n">
         <f aca="false">D39*D43/100</f>
-        <v>821.2943376</v>
+        <v>139.2</v>
       </c>
       <c r="H43" s="62" t="s">
         <v>53</v>
@@ -4763,7 +4794,7 @@
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="63" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C44" s="63"/>
       <c r="D44" s="1" t="n">
@@ -4777,7 +4808,7 @@
       </c>
       <c r="G44" s="88" t="n">
         <f aca="false">D39*D44/100</f>
-        <v>4106.471688</v>
+        <v>696</v>
       </c>
       <c r="H44" s="62" t="s">
         <v>53</v>
@@ -4786,7 +4817,7 @@
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="68" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C45" s="68"/>
       <c r="D45" s="42" t="n">
@@ -4800,7 +4831,7 @@
       </c>
       <c r="G45" s="84" t="n">
         <f aca="false">D39*D45/100</f>
-        <v>821.2943376</v>
+        <v>139.2</v>
       </c>
       <c r="H45" s="62" t="s">
         <v>53</v>
@@ -4809,17 +4840,17 @@
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="63" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C46" s="63"/>
       <c r="D46" s="1" t="n">
         <v>100</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="G46" s="88" t="n">
         <f aca="false">D46</f>
@@ -4830,17 +4861,17 @@
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="68" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C47" s="68"/>
       <c r="D47" s="42" t="n">
         <v>2</v>
       </c>
       <c r="E47" s="42" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="F47" s="42" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="G47" s="84" t="n">
         <f aca="false">D47*G11</f>
@@ -4862,7 +4893,7 @@
       <c r="F48" s="89"/>
       <c r="G48" s="90" t="n">
         <f aca="false">SUM(G41:G47)</f>
-        <v>20169.0294752293</v>
+        <v>3639.35154935185</v>
       </c>
       <c r="H48" s="91" t="s">
         <v>53</v>
@@ -4893,7 +4924,7 @@
       <c r="H50" s="94"/>
       <c r="I50" s="95" t="n">
         <f aca="false">D39-G48</f>
-        <v>61960.4042847707</v>
+        <v>10280.6484506482</v>
       </c>
       <c r="J50" s="79" t="s">
         <v>43</v>
@@ -5108,7 +5139,7 @@
       <c r="H64" s="94"/>
       <c r="I64" s="95" t="n">
         <f aca="false">I50+D56-D62</f>
-        <v>60860.4042847707</v>
+        <v>9180.64845064815</v>
       </c>
       <c r="J64" s="79" t="s">
         <v>43</v>
@@ -5141,7 +5172,7 @@
       <c r="G67" s="103"/>
       <c r="H67" s="104" t="n">
         <f aca="false">I64/D11/F15*1000</f>
-        <v>1482.06073020345</v>
+        <v>1319.05868543795</v>
       </c>
       <c r="I67" s="105" t="s">
         <v>46</v>

</xml_diff>